<commit_message>
update blood pressure descr 4be14c0c4cb4219f6130e9d8162b30af043c0f60
</commit_message>
<xml_diff>
--- a/nr-add-profile-list/ig/StructureDefinition-fr-core-observation-bp.xlsx
+++ b/nr-add-profile-list/ig/StructureDefinition-fr-core-observation-bp.xlsx
@@ -45,7 +45,7 @@
     <t>Title</t>
   </si>
   <si>
-    <t>FR Core Observation Bp Profile</t>
+    <t>FR Core Observation Blood Pressure Profile</t>
   </si>
   <si>
     <t>Status</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2024-03-21T10:58:03+00:00</t>
+    <t>2024-03-21T10:59:21+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -84,8 +84,8 @@
     <t>Description</t>
   </si>
   <si>
-    <t>French profil Blood pressure panel with all children optional - This is a component observation. It has no value in Observation.valueQuantity and contains at least one component (systolic and/or diastolic and/or mean).
-Profil français de pression artérielle avec tous les éléments fils optionnels. Il s'agit d'une Observation avec l'élément Observation.valueQuantity n'est pas renseigné et qui contient au moins un composant Pression systolique, Pression diastolique, Pression moyenne.</t>
+    <t>French profile for blood pressure.
+Profil français de la pression artérielle. Profil basé sur le profil bp d'HL7</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>